<commit_message>
feat: complete PRD-097 workspace onboarding
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..096已完成，下一项PRD-097。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..097已完成，下一项PRD-098。</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6572,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: add enterprise domain sso login discovery
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..097已完成，下一项PRD-098。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..114已完成，下一项PRD-115。</t>
         </is>
       </c>
     </row>
@@ -6703,7 +6703,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -6838,7 +6838,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -6972,7 +6972,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -7368,7 +7368,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -7638,7 +7638,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -7905,7 +7905,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -8039,7 +8039,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -8170,7 +8170,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -8435,7 +8435,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(identity): complete PRD-115 SCIM lifecycle
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..114已完成，下一项PRD-115。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..115已完成，下一项PRD-116。</t>
         </is>
       </c>
     </row>
@@ -8969,7 +8969,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(identity): complete PRD-116 identity security
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..115已完成，下一项PRD-116。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..116已完成，下一项PRD-117。</t>
         </is>
       </c>
     </row>
@@ -9101,7 +9101,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(providers): complete PRD-119 catalog compliance
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..116已完成，下一项PRD-117。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..119已完成，下一项PRD-120。</t>
         </is>
       </c>
     </row>
@@ -9501,7 +9501,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-120 device identity
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -31,7 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_里程碑门禁'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_风险与决策'!$A$1:$G$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10_角色页面矩阵'!$A$1:$F$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11_现有导航处置'!$A$1:$J$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11_现有导航处置'!$A$1:$J$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..119已完成，下一项PRD-120。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..120已完成，下一项PRD-121。</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>源码63项：44项企业Gateway保留，12项拆为独立平台/企业投影，5项完全迁入SaaS平台，1项迁到GlobalAccount壳层，1项退出登录后产品UI；不得只隐藏菜单，DOM、预取、API和数据owner必须同步切换。</t>
+          <t>源码64项：45项企业Gateway保留，12项拆为独立平台/企业投影，5项完全迁入SaaS平台，1项迁到GlobalAccount壳层，1项退出登录后产品UI；不得只隐藏菜单，DOM、预取、API和数据owner必须同步切换。</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2849,47 +2849,47 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>adapter-specs</t>
+          <t>private-gateways</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Adapter 规范</t>
+          <t>私有 Gateway</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>迁出企业</t>
+          <t>企业保留并归组</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>平台Provider工程台；企业Provider详情另建兼容摘要</t>
+          <t>客户自有Edge Deployment</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>owner/admin管理；developer/security_admin按权限只读</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>platform_provider_engineer/platform_security/release_manager</t>
+          <t>platform_ops只看独立Fleet脱敏投影</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>GET /adapter-specs；POST /internal/adapter-specs/{tenant_id}/activate；provider_adapter_catalog_activations</t>
+          <t>GET/POST /edge/deployments、/edge/registrations、/edge/deployments/{id}/revoke；edge_deployments及设备身份表</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>PRD-143/147</t>
+          <t>PRD-120..130/146</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>企业旧规范导航、DOM、预取和API归零；兼容摘要由Provider详情独立鉴权，不暴露内部schema、构建信息或发布权限</t>
+          <t>Workspace与Platform使用独立Session/API/DTO；注册材料、设备私钥、本地Secret和业务正文不得进入平台投影</t>
         </is>
       </c>
     </row>
@@ -2901,12 +2901,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>adapter-contract-runs</t>
+          <t>adapter-specs</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>CI 测试报告</t>
+          <t>Adapter 规范</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>平台Provider工程台</t>
+          <t>平台Provider工程台；企业Provider详情另建兼容摘要</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>GET /adapter-contract-runs及/{id}；POST /internal/tenants/{tenant_id}/adapter-contract-runs；runs/cases/outbox</t>
+          <t>GET /adapter-specs；POST /internal/adapter-specs/{tenant_id}/activate；provider_adapter_catalog_activations</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Runner、case详情和构建路径不进入企业DTO；企业兼容结论改在Provider详情提供；旧run/outbox水位保真</t>
+          <t>企业旧规范导航、DOM、预取和API归零；兼容摘要由Provider详情独立鉴权，不暴露内部schema、构建信息或发布权限</t>
         </is>
       </c>
     </row>
@@ -2953,47 +2953,47 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>provider-health</t>
+          <t>adapter-contract-runs</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Provider 状态</t>
+          <t>CI 测试报告</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>平台/企业拆分</t>
+          <t>迁出企业</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>本企业Provider健康；平台全局Provider/Cell健康</t>
+          <t>平台Provider工程台</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/security_admin/viewer按授权</t>
+          <t>无</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>platform_ops/platform_security/platform_support只读脱敏</t>
+          <t>platform_provider_engineer/platform_security/release_manager</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>GET /provider-health、POST /providers/{id}/probe；真实调用与探测事实</t>
+          <t>GET /adapter-contract-runs及/{id}；POST /internal/tenants/{tenant_id}/adapter-contract-runs；runs/cases/outbox</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>PRD-109/112/119/143/145</t>
+          <t>PRD-143/147</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>企业只见自身Endpoint/调用；平台聚合不得泄漏业务正文或Secret</t>
+          <t>Runner、case详情和构建路径不进入企业DTO；企业兼容结论改在Provider详情提供；旧run/outbox水位保真</t>
         </is>
       </c>
     </row>
@@ -3005,47 +3005,47 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>error-maps</t>
+          <t>provider-health</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>错误码管理</t>
+          <t>Provider 状态</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>平台/企业拆分并降级</t>
+          <t>平台/企业拆分</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>平台内置目录；企业受限覆盖</t>
+          <t>本企业Provider健康；平台全局Provider/Cell健康</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer高级入口</t>
+          <t>owner/admin/developer/security_admin/viewer按授权</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>platform_provider_engineer/platform_security/release_manager</t>
+          <t>platform_ops/platform_security/platform_support只读脱敏</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>GET/POST/PATCH /error-maps；builtin catalog、maps、versions、heads、events、facts</t>
+          <t>GET /provider-health、POST /providers/{id}/probe；真实调用与探测事实</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>PRD-143/147</t>
+          <t>PRD-109/112/119/143/145</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>企业不能改内置规则；覆盖只作用本Workspace且每个失败请求可解释追踪</t>
+          <t>企业只见自身Endpoint/调用；平台聚合不得泄漏业务正文或Secret</t>
         </is>
       </c>
     </row>
@@ -3057,47 +3057,47 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>models</t>
+          <t>error-maps</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>模型目录</t>
+          <t>错误码管理</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>平台/企业拆分并降级</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>企业可用模型</t>
+          <t>平台内置目录；企业受限覆盖</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer；viewer按授权只读</t>
+          <t>owner/admin/developer高级入口</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>平台Provider目录仅提供发布源</t>
+          <t>platform_provider_engineer/platform_security/release_manager</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>GET/POST/PATCH /models；模型owner保留tenant_id</t>
+          <t>GET/POST/PATCH /error-maps；builtin catalog、maps、versions、heads、events、facts</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>PRD-119/146</t>
+          <t>PRD-143/147</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>企业选择并治理自身可用模型；平台目录更新不能自动扩权</t>
+          <t>企业不能改内置规则；覆盖只作用本Workspace且每个失败请求可解释追踪</t>
         </is>
       </c>
     </row>
@@ -3109,12 +3109,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>model-aliases</t>
+          <t>models</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>模型别名</t>
+          <t>模型目录</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -3124,32 +3124,32 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>稳定业务模型别名</t>
+          <t>企业可用模型</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer按权限</t>
+          <t>owner/admin/developer；viewer按授权只读</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>平台Provider目录仅提供发布源</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>现有routing.read、model_aliases模块</t>
+          <t>GET/POST/PATCH /models；模型owner保留tenant_id</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>PRD-101/108/146</t>
+          <t>PRD-119/146</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>别名、环境和路由均绑定Workspace，切换可回滚</t>
+          <t>企业选择并治理自身可用模型；平台目录更新不能自动扩权</t>
         </is>
       </c>
     </row>
@@ -3161,12 +3161,12 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>routing-policies</t>
+          <t>model-aliases</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>路由策略</t>
+          <t>模型别名</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -3176,12 +3176,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>企业模型路由</t>
+          <t>稳定业务模型别名</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer按权限；auditor只读</t>
+          <t>owner/admin/developer按权限</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>现有routing.read及固定/成本/可用性路由</t>
+          <t>现有routing.read、model_aliases模块</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>后端准入与签名快照生效；前端隐藏不构成权限</t>
+          <t>别名、环境和路由均绑定Workspace，切换可回滚</t>
         </is>
       </c>
     </row>
@@ -3213,12 +3213,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>model-quality-scores</t>
+          <t>routing-policies</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>模型评分</t>
+          <t>路由策略</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -3228,32 +3228,32 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>企业模型质量与SLO</t>
+          <t>企业模型路由</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/viewer按授权</t>
+          <t>owner/admin/developer按权限；auditor只读</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>platform_ops只看平台运行聚合</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>现有model_quality.read、真实成功率/延迟与人工先验</t>
+          <t>现有routing.read及固定/成本/可用性路由</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>PRD-109/119/146</t>
+          <t>PRD-101/108/146</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>企业评分不成为平台客户健康或增长画像；聚合最小化</t>
+          <t>后端准入与签名快照生效；前端隐藏不构成权限</t>
         </is>
       </c>
     </row>
@@ -3265,12 +3265,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>experiments</t>
+          <t>model-quality-scores</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>模型评测</t>
+          <t>模型评分</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -3280,49 +3280,49 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>企业模型评测与A/B</t>
+          <t>企业模型质量与SLO</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer按权限；auditor只读</t>
+          <t>owner/admin/developer/viewer按授权</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_ops只看平台运行聚合</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>现有experiment.read及不可变实验配置/结果</t>
+          <t>现有model_quality.read、真实成功率/延迟与人工先验</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>PRD-101/106/146</t>
+          <t>PRD-109/119/146</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>分流、停止、用量和成本都绑定本Workspace并可审计</t>
+          <t>企业评分不成为平台客户健康或增长画像；聚合最小化</t>
         </is>
       </c>
     </row>
     <row r="24" ht="108" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>调用与成本</t>
+          <t>配置</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>projects</t>
+          <t>experiments</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>项目与应用</t>
+          <t>模型评测</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -3332,12 +3332,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>企业项目与应用</t>
+          <t>企业模型评测与A/B</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer；finance/security按范围只读</t>
+          <t>owner/admin/developer按权限；auditor只读</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -3347,17 +3347,17 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>现有project.read；Project/Application为Key、日志、预算归属</t>
+          <t>现有experiment.read及不可变实验配置/结果</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>PRD-094/146</t>
+          <t>PRD-101/106/146</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>所有对象带tenant_id；职能角色只见授权项目</t>
+          <t>分流、停止、用量和成本都绑定本Workspace并可审计</t>
         </is>
       </c>
     </row>
@@ -3369,12 +3369,12 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>virtual-keys</t>
+          <t>projects</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Virtual Key</t>
+          <t>项目与应用</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -3384,32 +3384,32 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>业务调用凭据</t>
+          <t>企业项目与应用</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer按权限</t>
+          <t>owner/admin/developer；finance/security按范围只读</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>platform_support与平台运营均不可读Secret</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>现有virtual_key.read及Key生命周期</t>
+          <t>现有project.read；Project/Application为Key、日志、预算归属</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>PRD-100/118/146</t>
+          <t>PRD-094/146</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>只显示一次的Secret不入日志；撤销、失败、用量和成本可追踪</t>
+          <t>所有对象带tenant_id；职能角色只见授权项目</t>
         </is>
       </c>
     </row>
@@ -3421,47 +3421,47 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>usage</t>
+          <t>virtual-keys</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>用量与成本</t>
+          <t>Virtual Key</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>企业保留；平台另建计量</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>企业技术用量与内部成本</t>
+          <t>业务调用凭据</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/finance_admin/auditor/viewer按字段</t>
+          <t>owner/admin/developer按权限</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>platform_billing只见平台商业计量</t>
+          <t>platform_support与平台运营均不可读Secret</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>GET /usage/*；Usage与价格快照</t>
+          <t>现有virtual_key.read及Key生命周期</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>PRD-099/122/144/146</t>
+          <t>PRD-100/118/146</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>平台计量与企业业务用量字段分域；成功失败取消重试均可追踪</t>
+          <t>只显示一次的Secret不入日志；撤销、失败、用量和成本可追踪</t>
         </is>
       </c>
     </row>
@@ -3473,47 +3473,47 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>finops-ledger</t>
+          <t>usage</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>FinOps 账本</t>
+          <t>用量与成本</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>企业保留；平台账本拆分</t>
+          <t>企业保留；平台另建计量</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>企业内部FinOps</t>
+          <t>企业技术用量与内部成本</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>owner/finance_admin；auditor只读</t>
+          <t>owner/admin/developer/finance_admin/auditor/viewer按字段</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>platform_billing仅平台商业账</t>
+          <t>platform_billing只见平台商业计量</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>GET/POST /finops/ledger；不可变分录与价格证据</t>
+          <t>GET /usage/*；Usage与价格快照</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>PRD-099/104/144/146</t>
+          <t>PRD-099/122/144/146</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>企业内部成本调整与平台收费分录不能互相写入或冒充</t>
+          <t>平台计量与企业业务用量字段分域；成功失败取消重试均可追踪</t>
         </is>
       </c>
     </row>
@@ -3525,47 +3525,47 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>model-prices</t>
+          <t>finops-ledger</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>模型价格</t>
+          <t>FinOps 账本</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>平台/企业拆分</t>
+          <t>企业保留；平台账本拆分</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>平台官方建议价；企业BYOK成本价</t>
+          <t>企业内部FinOps</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>owner/finance_admin；developer只读可用价格</t>
+          <t>owner/finance_admin；auditor只读</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>platform_billing/release_manager</t>
+          <t>platform_billing仅平台商业账</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>GET/POST /model-prices；历史/当前/未来价格与Usage快照</t>
+          <t>GET/POST /finops/ledger；不可变分录与价格证据</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>PRD-098/119/144/147</t>
+          <t>PRD-099/104/144/146</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>价格来源和版本明确；企业不能发布平台价，平台不能改企业私有成本</t>
+          <t>企业内部成本调整与平台收费分录不能互相写入或冒充</t>
         </is>
       </c>
     </row>
@@ -3577,47 +3577,47 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>response-cache</t>
+          <t>model-prices</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>响应缓存</t>
+          <t>模型价格</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>企业保留并入高级配置</t>
+          <t>平台/企业拆分</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>模型别名/路由详情的缓存策略</t>
+          <t>平台官方建议价；企业BYOK成本价</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/security_admin按权限</t>
+          <t>owner/finance_admin；developer只读可用价格</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_billing/release_manager</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>现有response_cache.read及按模型别名的可选能力</t>
+          <t>GET/POST /model-prices；历史/当前/未来价格与Usage快照</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>PRD-101/108/117/146</t>
+          <t>PRD-098/119/144/147</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>不占普通一级导航；默认不缓存正文；租户、模型、保留和计费owner一致</t>
+          <t>价格来源和版本明确；企业不能发布平台价，平台不能改企业私有成本</t>
         </is>
       </c>
     </row>
@@ -3629,47 +3629,47 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>plans</t>
+          <t>response-cache</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>套餐管理</t>
+          <t>响应缓存</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>平台/企业拆分并改名</t>
+          <t>企业保留并入高级配置</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>平台套餐目录；企业订阅摘要</t>
+          <t>模型别名/路由详情的缓存策略</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>owner/finance_admin只读本Workspace订阅</t>
+          <t>owner/admin/developer/security_admin按权限</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>platform_owner/platform_billing</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>GET/PATCH /plans；plan/trial/quota事实</t>
+          <t>现有response_cache.read及按模型别名的可选能力</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>PRD-098/144/147</t>
+          <t>PRD-101/108/117/146</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>企业无套餐目录写入；Entitlement后端生效且回滚不扩大权益</t>
+          <t>不占普通一级导航；默认不缓存正文；租户、模型、保留和计费owner一致</t>
         </is>
       </c>
     </row>
@@ -3681,47 +3681,47 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>quota-buckets</t>
+          <t>plans</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>额度管理</t>
+          <t>套餐管理</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>企业保留；平台发放拆分</t>
+          <t>平台/企业拆分并改名</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>企业内部额度分配与消费</t>
+          <t>平台套餐目录；企业订阅摘要</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/finance_admin；developer只读自身</t>
+          <t>owner/finance_admin只读本Workspace订阅</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>platform_billing管理Entitlement上限而非企业分配</t>
+          <t>platform_owner/platform_billing</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>GET /quota-buckets；POST /quota-adjustments；四类额度及消费</t>
+          <t>GET/PATCH /plans；plan/trial/quota事实</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>PRD-098/099/144/146</t>
+          <t>PRD-098/144/147</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>平台权益上限和企业Project/Key额度分别授权、共同失败关闭</t>
+          <t>企业无套餐目录写入；Entitlement后端生效且回滚不扩大权益</t>
         </is>
       </c>
     </row>
@@ -3733,47 +3733,47 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>billing-disputes</t>
+          <t>quota-buckets</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>账单争议</t>
+          <t>额度管理</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>平台/企业拆分</t>
+          <t>企业保留；平台发放拆分</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>企业争议申请；平台争议裁决</t>
+          <t>企业内部额度分配与消费</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>owner/finance_admin提交和查看自身</t>
+          <t>owner/admin/finance_admin；developer只读自身</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>platform_billing裁决；platform_support协作但不裁决</t>
+          <t>platform_billing管理Entitlement上限而非企业分配</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>GET/POST/PATCH /billing-disputes；0073争议/调整状态机</t>
+          <t>GET /quota-buckets；POST /quota-adjustments；四类额度及消费</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>PRD-104/132/144/147</t>
+          <t>PRD-098/099/144/146</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>申请人不能裁决；金额调整不可变、双审批、统一审计和request_id</t>
+          <t>平台权益上限和企业Project/Key额度分别授权、共同失败关闭</t>
         </is>
       </c>
     </row>
@@ -3785,47 +3785,47 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>budgets</t>
+          <t>billing-disputes</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>预算中心</t>
+          <t>账单争议</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>平台/企业拆分</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>企业多级预算</t>
+          <t>企业争议申请；平台争议裁决</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/finance_admin；developer/auditor按范围只读</t>
+          <t>owner/finance_admin提交和查看自身</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_billing裁决；platform_support协作但不裁决</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>GET/POST/PATCH /budgets及/budget-status</t>
+          <t>GET/POST/PATCH /billing-disputes；0073争议/调整状态机</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>PRD-099/106/146</t>
+          <t>PRD-104/132/144/147</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>tenant/Project/Key预算后端准入；失败、阻断、审批和成本可追踪</t>
+          <t>申请人不能裁决；金额调整不可变、双审批、统一审计和request_id</t>
         </is>
       </c>
     </row>
@@ -3837,99 +3837,99 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>cost-anomalies</t>
+          <t>budgets</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>成本异常</t>
+          <t>预算中心</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>企业保留；平台另建商业异常</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>企业BYOK与内部成本异常</t>
+          <t>企业多级预算</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>owner/finance_admin/security_admin；auditor只读</t>
+          <t>owner/admin/finance_admin；developer/auditor按范围只读</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>platform_billing只看平台收费异常</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>GET/PATCH /cost-anomalies；runs/anomalies/actions/temporary overrides</t>
+          <t>GET/POST/PATCH /budgets及/budget-status</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>PRD-099/106/109/144/146</t>
+          <t>PRD-099/106/146</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>企业异常不泄漏到其他客户；平台异常不得获得Prompt/Response</t>
+          <t>tenant/Project/Key预算后端准入；失败、阻断、审批和成本可追踪</t>
         </is>
       </c>
     </row>
     <row r="35" ht="108" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>安全与治理</t>
+          <t>调用与成本</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>policies</t>
+          <t>cost-anomalies</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>策略管理</t>
+          <t>成本异常</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>企业保留；平台另建商业异常</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>企业治理策略</t>
+          <t>企业BYOK与内部成本异常</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin；developer/auditor只读授权范围</t>
+          <t>owner/finance_admin/security_admin；auditor只读</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_billing只看平台收费异常</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>现有policy.read及受限DSL</t>
+          <t>GET/PATCH /cost-anomalies；runs/anomalies/actions/temporary overrides</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>PRD-108/117/146</t>
+          <t>PRD-099/106/109/144/146</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>策略owner、版本、发布和回滚可审计；失效按安全类别失败关闭</t>
+          <t>企业异常不泄漏到其他客户；平台异常不得获得Prompt/Response</t>
         </is>
       </c>
     </row>
@@ -3941,27 +3941,27 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>policy-simulator</t>
+          <t>policies</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>策略模拟器</t>
+          <t>策略管理</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>企业保留并归高级工具</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>企业策略预演</t>
+          <t>企业治理策略</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin/developer按权限</t>
+          <t>owner/admin/security_admin；developer/auditor只读授权范围</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -3971,17 +3971,17 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>现有policy.simulate；不调用真实Provider</t>
+          <t>现有policy.read及受限DSL</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>PRD-108/146</t>
+          <t>PRD-108/117/146</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>预演不能改变生产事实；输入正文不进入日志或验收证据</t>
+          <t>策略owner、版本、发布和回滚可审计；失效按安全类别失败关闭</t>
         </is>
       </c>
     </row>
@@ -3993,27 +3993,27 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>policy-snapshots</t>
+          <t>policy-simulator</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>策略发布</t>
+          <t>策略模拟器</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>企业保留并归高级工具</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>企业策略版本与回滚</t>
+          <t>企业策略预演</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin；auditor只读</t>
+          <t>owner/admin/security_admin/developer按权限</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -4023,17 +4023,17 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>现有policy.read及不可变快照</t>
+          <t>现有policy.simulate；不调用真实Provider</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>PRD-108/121/146</t>
+          <t>PRD-108/146</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>签名、generation、LKG和动态撤权合同生效</t>
+          <t>预演不能改变生产事实；输入正文不进入日志或验收证据</t>
         </is>
       </c>
     </row>
@@ -4045,47 +4045,47 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>policy-templates</t>
+          <t>policy-snapshots</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>策略模板库</t>
+          <t>策略发布</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>平台/企业拆分</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>平台模板目录；企业应用与覆盖</t>
+          <t>企业策略版本与回滚</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin应用；auditor只读</t>
+          <t>owner/admin/security_admin；auditor只读</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>platform_security/platform_compliance/release_manager发布</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>GET /policy-templates；POST /policy-templates/{policy_template_id}/apply；内置模板、适配和绑定事实</t>
+          <t>现有policy.read及不可变快照</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>PRD-117/119/143/146</t>
+          <t>PRD-108/121/146</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>企业不能篡改内置模板；套用产生tenant-scoped版本并可回滚</t>
+          <t>签名、generation、LKG和动态撤权合同生效</t>
         </is>
       </c>
     </row>
@@ -4097,47 +4097,47 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>dlp-rules</t>
+          <t>policy-templates</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>DLP 规则</t>
+          <t>策略模板库</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>平台/企业拆分</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>企业DLP</t>
+          <t>平台模板目录；企业应用与覆盖</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin；auditor只读</t>
+          <t>owner/admin/security_admin应用；auditor只读</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_security/platform_compliance/release_manager发布</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>现有dlp.read及log_only/block规则</t>
+          <t>GET /policy-templates；POST /policy-templates/{policy_template_id}/apply；内置模板、适配和绑定事实</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>PRD-108/117/146</t>
+          <t>PRD-117/119/143/146</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>Provider前失败关闭；命中证据不保存Prompt/Response正文</t>
+          <t>企业不能篡改内置模板；套用产生tenant-scoped版本并可回滚</t>
         </is>
       </c>
     </row>
@@ -4149,27 +4149,27 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>intent-security</t>
+          <t>dlp-rules</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>敏感意图分类</t>
+          <t>DLP 规则</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>企业保留并降级</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>安全管理员测试工具</t>
+          <t>企业DLP</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>security_admin；owner/admin按权限</t>
+          <t>owner/admin/security_admin；auditor只读</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -4179,17 +4179,17 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>现有intent_risk.classify；本地轻量规则</t>
+          <t>现有dlp.read及log_only/block规则</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>PRD-110/146</t>
+          <t>PRD-108/117/146</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>不作为普通导航；结果不含原文/命中片段；限流与审计</t>
+          <t>Provider前失败关闭；命中证据不保存Prompt/Response正文</t>
         </is>
       </c>
     </row>
@@ -4201,47 +4201,47 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>session-risks</t>
+          <t>intent-security</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>高危会话</t>
+          <t>敏感意图分类</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>企业保留并降级</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>企业会话风险处置</t>
+          <t>安全管理员测试工具</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin；auditor只读</t>
+          <t>security_admin；owner/admin按权限</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>platform_support仅经SupportGrant看固定摘要</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>现有session_risk.read及冻结/审批记录</t>
+          <t>现有intent_risk.classify；本地轻量规则</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>PRD-116/137/146</t>
+          <t>PRD-110/146</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>处置绑定Workspace并动态撤权；平台默认看不到会话正文</t>
+          <t>不作为普通导航；结果不含原文/命中片段；限流与审计</t>
         </is>
       </c>
     </row>
@@ -4253,12 +4253,12 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>output-safety</t>
+          <t>session-risks</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>输出安全事件</t>
+          <t>高危会话</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>企业输出安全</t>
+          <t>企业会话风险处置</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -4278,22 +4278,22 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>platform_security只看脱敏聚合</t>
+          <t>platform_support仅经SupportGrant看固定摘要</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>现有request_log.read的阻断/扫描事实</t>
+          <t>现有session_risk.read及冻结/审批记录</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>PRD-108/109/117/146</t>
+          <t>PRD-116/137/146</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>正文默认不持久化；事件含owner、code、request_id而非输出明文</t>
+          <t>处置绑定Workspace并动态撤权；平台默认看不到会话正文</t>
         </is>
       </c>
     </row>
@@ -4305,12 +4305,12 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>webhooks</t>
+          <t>output-safety</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Webhook 设置</t>
+          <t>输出安全事件</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -4320,32 +4320,32 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>企业治理事件订阅</t>
+          <t>企业输出安全</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin</t>
+          <t>owner/admin/security_admin；auditor只读</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_security只看脱敏聚合</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>现有webhook.manage、Endpoint与签名Secret</t>
+          <t>现有request_log.read的阻断/扫描事实</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>PRD-105/133/146</t>
+          <t>PRD-108/109/117/146</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>签名Secret只显示一次；SSRF、重放、出站ACL和审计通过</t>
+          <t>正文默认不持久化；事件含owner、code、request_id而非输出明文</t>
         </is>
       </c>
     </row>
@@ -4357,22 +4357,22 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>webhook-dead-letters</t>
+          <t>webhooks</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Webhook 死信</t>
+          <t>Webhook 设置</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>企业保留并降级</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>企业高级运维入口</t>
+          <t>企业治理事件订阅</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -4387,17 +4387,17 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>现有webhook.manage、持久死信与安全重放</t>
+          <t>现有webhook.manage、Endpoint与签名Secret</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>PRD-106/146</t>
+          <t>PRD-105/133/146</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>不默认出现在普通导航；重放幂等、限次且不能修改冻结payload</t>
+          <t>签名Secret只显示一次；SSRF、重放、出站ACL和审计通过</t>
         </is>
       </c>
     </row>
@@ -4409,99 +4409,99 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>audit-logs</t>
+          <t>webhook-dead-letters</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>审计日志</t>
+          <t>Webhook 死信</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>企业保留；平台审计拆分</t>
+          <t>企业保留并降级</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>企业不可变审计</t>
+          <t>企业高级运维入口</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin/legal_admin/auditor</t>
+          <t>owner/admin/security_admin</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>各platform_*只见自身平台审计；支持受Grant限制</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>现有audit.read及不可变audit_logs</t>
+          <t>现有webhook.manage、持久死信与安全重放</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>PRD-095/117/135/145/146</t>
+          <t>PRD-106/146</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>平台和企业审计域分离；Key/Token/Prompt/Response不入证据</t>
+          <t>不默认出现在普通导航；重放幂等、限次且不能修改冻结payload</t>
         </is>
       </c>
     </row>
     <row r="46" ht="108" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>调用与成本</t>
+          <t>安全与治理</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>request-logs</t>
+          <t>audit-logs</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>调用日志</t>
+          <t>审计日志</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>企业保留；平台审计拆分</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>企业调用可观测性</t>
+          <t>企业不可变审计</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/security_admin/auditor/viewer按字段</t>
+          <t>owner/admin/security_admin/legal_admin/auditor</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>platform_support仅JIT白名单摘要</t>
+          <t>各platform_*只见自身平台审计；支持受Grant限制</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>现有request_log.read及分页/trace</t>
+          <t>现有audit.read及不可变audit_logs</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>PRD-109/117/146</t>
+          <t>PRD-095/117/135/145/146</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>只加载当前页；正文/Secret不记录；失败与用量成本可关联</t>
+          <t>平台和企业审计域分离；Key/Token/Prompt/Response不入证据</t>
         </is>
       </c>
     </row>
@@ -4513,27 +4513,27 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>request-explanations</t>
+          <t>request-logs</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>请求解释</t>
+          <t>调用日志</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>企业保留并入日志详情</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>调用日志详情的路由/策略/成本解释</t>
+          <t>企业调用可观测性</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/security_admin/finance_admin/auditor按字段</t>
+          <t>owner/admin/developer/security_admin/auditor/viewer按字段</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -4543,17 +4543,17 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>现有request_explanation.read</t>
+          <t>现有request_log.read及分页/trace</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>PRD-108/109/146</t>
+          <t>PRD-109/117/146</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>不占普通一级导航；解释字段按职能裁剪；不能通过解释恢复Prompt/Response或Key</t>
+          <t>只加载当前页；正文/Secret不记录；失败与用量成本可关联</t>
         </is>
       </c>
     </row>
@@ -4565,99 +4565,99 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>feedback-summary</t>
+          <t>request-explanations</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>反馈报表</t>
+          <t>请求解释</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>企业保留并入日志详情</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>企业模型反馈与质量</t>
+          <t>调用日志详情的路由/策略/成本解释</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/viewer按权限</t>
+          <t>owner/admin/developer/security_admin/finance_admin/auditor按字段</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>platform_customer_success只读脱敏采用摘要，不读反馈正文</t>
+          <t>platform_support仅JIT白名单摘要</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>现有feedback.use及聚合报表</t>
+          <t>现有request_explanation.read</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>PRD-109/140/146</t>
+          <t>PRD-108/109/146</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>企业反馈不成为平台个体画像；跨域只传最小聚合</t>
+          <t>不占普通一级导航；解释字段按职能裁剪；不能通过解释恢复Prompt/Response或Key</t>
         </is>
       </c>
     </row>
     <row r="49" ht="108" customHeight="1">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>开发者</t>
+          <t>调用与成本</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>quickstart</t>
+          <t>feedback-summary</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>快速开始</t>
+          <t>反馈报表</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>企业保留并任务化</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>角色化初始化向导</t>
+          <t>企业模型反馈与质量</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer</t>
+          <t>owner/admin/developer/viewer按权限</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>platform_support只协助脱敏状态</t>
+          <t>platform_customer_success只读脱敏采用摘要，不读反馈正文</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>现有developer_portal.read；静态步骤改为真实后端完成事实</t>
+          <t>现有feedback.use及聚合报表</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>PRD-097/146</t>
+          <t>PRD-109/140/146</t>
         </is>
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>步骤可点击、可查看证据、失败可恢复，不以假数据标记已完成</t>
+          <t>企业反馈不成为平台个体画像；跨域只传最小聚合</t>
         </is>
       </c>
     </row>
@@ -4669,47 +4669,47 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>sdk-examples</t>
+          <t>quickstart</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>SDK 示例</t>
+          <t>快速开始</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>企业保留并入开发者中心</t>
+          <t>企业保留并任务化</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>开发者中心的SDK示例</t>
+          <t>角色化初始化向导</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>developer；owner/admin按需</t>
+          <t>owner/admin/developer</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_support只协助脱敏状态</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>现有developer_portal.read及示例</t>
+          <t>现有developer_portal.read；静态步骤改为真实后端完成事实</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>PRD-133/146</t>
+          <t>PRD-097/146</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>不占普通一级导航；示例使用占位值，不含真实Key；与N/N-1合同一致</t>
+          <t>步骤可点击、可查看证据、失败可恢复，不以假数据标记已完成</t>
         </is>
       </c>
     </row>
@@ -4721,12 +4721,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>migration-guide</t>
+          <t>sdk-examples</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>迁移指南</t>
+          <t>SDK 示例</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -4736,32 +4736,32 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>开发者中心的迁移兼容指南</t>
+          <t>开发者中心的SDK示例</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer</t>
+          <t>developer；owner/admin按需</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>platform_support可见公开内容</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>现有developer_portal.read；迁移平台兼容说明</t>
+          <t>现有developer_portal.read及示例</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>PRD-131/133/146</t>
+          <t>PRD-133/146</t>
         </is>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>不占普通一级导航；OpenRouter/硅基流动仅作为迁移兼容对象，不列为默认上游</t>
+          <t>不占普通一级导航；示例使用占位值，不含真实Key；与N/N-1合同一致</t>
         </is>
       </c>
     </row>
@@ -4773,12 +4773,12 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>api-docs</t>
+          <t>migration-guide</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>API 文档</t>
+          <t>迁移指南</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -4788,136 +4788,136 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>开发者中心的API文档</t>
+          <t>开发者中心的迁移兼容指南</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>developer；owner/admin按需</t>
+          <t>owner/admin/developer</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>platform_support只见公开合同</t>
+          <t>platform_support可见公开内容</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>现有console.basic.read；API合同与SDK版本</t>
+          <t>现有developer_portal.read；迁移平台兼容说明</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>PRD-133/146</t>
+          <t>PRD-131/133/146</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>不占普通一级导航；文档示例无Secret；错误码/request_id、版本和废弃期明确</t>
+          <t>不占普通一级导航；OpenRouter/硅基流动仅作为迁移兼容对象，不列为默认上游</t>
         </is>
       </c>
     </row>
     <row r="53" ht="108" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>帮助中心</t>
+          <t>开发者</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>competitor-comparison</t>
+          <t>api-docs</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>竞品对比</t>
+          <t>API 文档</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>迁出产品控制台</t>
+          <t>企业保留并入开发者中心</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>平台市场/销售内容或外部文档</t>
+          <t>开发者中心的API文档</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>developer；owner/admin按需</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>platform_growth/platform_channel只管理已审核内容</t>
+          <t>platform_support只见公开合同</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>当前主要为console-web静态render，无租户业务API</t>
+          <t>现有console.basic.read；API合同与SDK版本</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>PRD-141/146/147</t>
+          <t>PRD-133/146</t>
         </is>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>企业登录后产品UI不展示销售对比；迁移兼容说明仍可在迁移指南出现</t>
+          <t>不占普通一级导航；文档示例无Secret；错误码/request_id、版本和废弃期明确</t>
         </is>
       </c>
     </row>
     <row r="54" ht="108" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>开发者</t>
+          <t>帮助中心</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>enterprise-chat</t>
+          <t>competitor-comparison</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>企业 Chat</t>
+          <t>竞品对比</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>迁出产品控制台</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>企业AI应用</t>
+          <t>平台市场/销售内容或外部文档</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>获授权业务用户；配置由owner/admin/developer</t>
+          <t>无</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_growth/platform_channel只管理已审核内容</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>现有chat.use及企业会话owner</t>
+          <t>当前主要为console-web静态render，无租户业务API</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>PRD-116/117/146</t>
+          <t>PRD-141/146/147</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>会话和正文按租户策略处理；不同职能页面与动作不同</t>
+          <t>企业登录后产品UI不展示销售对比；迁移兼容说明仍可在迁移指南出现</t>
         </is>
       </c>
     </row>
@@ -4929,12 +4929,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>prompt-templates</t>
+          <t>enterprise-chat</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Prompt 模板</t>
+          <t>企业 Chat</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -4944,32 +4944,32 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>企业Prompt资产</t>
+          <t>企业AI应用</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer及获授权用户</t>
+          <t>获授权业务用户；配置由owner/admin/developer</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>platform_support无正文</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>现有prompt_template.read及企业模板库</t>
+          <t>现有chat.use及企业会话owner</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>PRD-117/146</t>
+          <t>PRD-116/117/146</t>
         </is>
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>Prompt不得进入日志或验收证据；版本/权限/审计绑定tenant</t>
+          <t>会话和正文按租户策略处理；不同职能页面与动作不同</t>
         </is>
       </c>
     </row>
@@ -4981,12 +4981,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>files</t>
+          <t>prompt-templates</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>文件处理</t>
+          <t>Prompt 模板</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>企业文件调用工具</t>
+          <t>企业Prompt资产</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -5011,121 +5011,121 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>现有file.read、提取与处理任务</t>
+          <t>现有prompt_template.read及企业模板库</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>PRD-117/122/146</t>
+          <t>PRD-117/146</t>
         </is>
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>文件正文、对象路径和提取文本受驻留/保留/DLP约束</t>
+          <t>Prompt不得进入日志或验收证据；版本/权限/审计绑定tenant</t>
         </is>
       </c>
     </row>
     <row r="57" ht="108" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>安全与治理</t>
+          <t>开发者</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>file-security</t>
+          <t>files</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>文件安全报告</t>
+          <t>文件处理</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>企业保留并入详情</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>文件详情与安全中心</t>
+          <t>企业文件调用工具</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/security_admin/developer/auditor按字段</t>
+          <t>owner/admin/developer及获授权用户</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>platform_security只看脱敏聚合</t>
+          <t>platform_support无正文</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>现有file.read、0066 outbox恢复事实</t>
+          <t>现有file.read、提取与处理任务</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>PRD-117/122/137/146</t>
+          <t>PRD-117/122/146</t>
         </is>
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>不占普通一级导航；不重复实现PRD-073；报告不含正文，outbox水位可恢复</t>
+          <t>文件正文、对象路径和提取文本受驻留/保留/DLP约束</t>
         </is>
       </c>
     </row>
     <row r="58" ht="108" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>开发者</t>
+          <t>安全与治理</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>batch-jobs</t>
+          <t>file-security</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>批处理任务</t>
+          <t>文件安全报告</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>企业保留</t>
+          <t>企业保留并入详情</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>企业异步批处理</t>
+          <t>文件详情与安全中心</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer；finance/auditor只读归属摘要</t>
+          <t>owner/admin/security_admin/developer/auditor按字段</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>platform_ops只看平台队列健康</t>
+          <t>platform_security只看脱敏聚合</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>现有batch.read、0067 Scheduler/Worker</t>
+          <t>现有file.read、0066 outbox恢复事实</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>PRD-106/113/146</t>
+          <t>PRD-117/122/137/146</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>job/lease/副作用均带tenant owner；企业看不到其他租户或平台队列内部</t>
+          <t>不占普通一级导航；不重复实现PRD-073；报告不含正文，outbox水位可恢复</t>
         </is>
       </c>
     </row>
@@ -5137,203 +5137,203 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>mcp-tools</t>
+          <t>batch-jobs</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>MCP 工具</t>
+          <t>批处理任务</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>企业保留并入开发者中心</t>
+          <t>企业保留</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>开发者中心的MCP治理</t>
+          <t>企业异步批处理</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/security_admin按权限</t>
+          <t>owner/admin/developer；finance/auditor只读归属摘要</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_ops只看平台队列健康</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>现有mcp.read及注册/权限/网络ACL</t>
+          <t>现有batch.read、0067 Scheduler/Worker</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>PRD-110/117/118/146</t>
+          <t>PRD-106/113/146</t>
         </is>
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>不占普通一级导航；工具scope、出站网络和机器身份最小授权；Secret不入日志</t>
+          <t>job/lease/副作用均带tenant owner；企业看不到其他租户或平台队列内部</t>
         </is>
       </c>
     </row>
     <row r="60" ht="108" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>租户治理</t>
+          <t>开发者</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>tenant-data-lifecycle</t>
+          <t>mcp-tools</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>数据管理</t>
+          <t>MCP 工具</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>企业保留并改名</t>
+          <t>企业保留并入开发者中心</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Workspace数据与隐私</t>
+          <t>开发者中心的MCP治理</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>owner/legal_admin/security_admin/auditor按动作</t>
+          <t>owner/admin/developer/security_admin按权限</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>platform_privacy只处理全局账号请求和最小队列</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>现有tenant_data.read、导出/删除/注销状态</t>
+          <t>现有mcp.read及注册/权限/网络ACL</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>PRD-117/134/146</t>
+          <t>PRD-110/117/118/146</t>
         </is>
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>复核tenant_data_states；导出/删除不允许平台支持绕过客户授权</t>
+          <t>不占普通一级导航；工具scope、出站网络和机器身份最小授权；Secret不入日志</t>
         </is>
       </c>
     </row>
     <row r="61" ht="108" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>开发者</t>
+          <t>租户治理</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>debug-console</t>
+          <t>tenant-data-lifecycle</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>OpenAI 调试台</t>
+          <t>数据管理</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>企业保留并降级</t>
+          <t>企业保留并改名</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>开发者高级工具</t>
+          <t>Workspace数据与隐私</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>developer；owner/admin按权限</t>
+          <t>owner/legal_admin/security_admin/auditor按动作</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>无</t>
+          <t>platform_privacy只处理全局账号请求和最小队列</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>现有debug_console.use；真实Gateway调用</t>
+          <t>现有tenant_data.read、导出/删除/注销状态</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>PRD-110/133/146</t>
+          <t>PRD-117/134/146</t>
         </is>
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>默认不向非开发角色展示；Key/Prompt/Response不进入日志或验收证据</t>
+          <t>复核tenant_data_states；导出/删除不允许平台支持绕过客户授权</t>
         </is>
       </c>
     </row>
     <row r="62" ht="108" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>系统</t>
+          <t>开发者</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>system-status</t>
+          <t>debug-console</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>系统状态</t>
+          <t>OpenAI 调试台</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>平台/企业拆分</t>
+          <t>企业保留并降级</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Workspace服务状态；平台SRE状态</t>
+          <t>开发者高级工具</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>owner/admin/developer/viewer按授权</t>
+          <t>developer；owner/admin按权限</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>platform_ops/platform_support/platform_owner</t>
+          <t>无</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>现有console.basic.read/provider status；平台另建Cell/Fleet/依赖状态</t>
+          <t>现有debug_console.use；真实Gateway调用</t>
         </is>
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>PRD-109/112/145</t>
+          <t>PRD-110/133/146</t>
         </is>
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>企业只见与自身相关的可操作状态；平台状态不暴露客户业务数据</t>
+          <t>默认不向非开发角色展示；Key/Prompt/Response不进入日志或验收证据</t>
         </is>
       </c>
     </row>
@@ -5345,47 +5345,47 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>language-settings</t>
+          <t>system-status</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>语言设置</t>
+          <t>系统状态</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>迁到全局账号壳层</t>
+          <t>平台/企业拆分</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>GlobalAccount偏好</t>
+          <t>Workspace服务状态；平台SRE状态</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>所有交互式账号本人</t>
+          <t>owner/admin/developer/viewer按授权</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>所有平台交互式账号本人</t>
+          <t>platform_ops/platform_support/platform_owner</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>现有user_preferences；不再作为tenant业务页面</t>
+          <t>现有console.basic.read/provider status；平台另建Cell/Fleet/依赖状态</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>PRD-091/105/145</t>
+          <t>PRD-109/112/145</t>
         </is>
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>语言不携带tenant角色、不改变权限；跨Workspace一致且可回退</t>
+          <t>企业只见与自身相关的可操作状态；平台状态不暴露客户业务数据</t>
         </is>
       </c>
     </row>
@@ -5397,52 +5397,104 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
+          <t>language-settings</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>语言设置</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>迁到全局账号壳层</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>GlobalAccount偏好</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>所有交互式账号本人</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>所有平台交互式账号本人</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>现有user_preferences；不再作为tenant业务页面</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>PRD-091/105/145</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>语言不携带tenant角色、不改变权限；跨Workspace一致且可回退</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="108" customHeight="1">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>系统</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
           <t>config-summary</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
         <is>
           <t>环境信息</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>平台/企业拆分并降级</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
+      <c r="E65" s="3" t="inlineStr">
         <is>
           <t>Deployment诊断；平台运行配置摘要</t>
         </is>
       </c>
-      <c r="F64" s="3" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
         <is>
           <t>owner/admin/developer高级入口；auditor只读脱敏</t>
         </is>
       </c>
-      <c r="G64" s="3" t="inlineStr">
+      <c r="G65" s="3" t="inlineStr">
         <is>
           <t>platform_ops/platform_security；support需Grant</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr">
+      <c r="H65" s="3" t="inlineStr">
         <is>
           <t>GET /internal/config/summary；当前system.config.read</t>
         </is>
       </c>
-      <c r="I64" s="3" t="inlineStr">
+      <c r="I65" s="3" t="inlineStr">
         <is>
           <t>PRD-109/120/125/145/147</t>
         </is>
       </c>
-      <c r="J64" s="3" t="inlineStr">
+      <c r="J65" s="3" t="inlineStr">
         <is>
           <t>普通用户不见环境变量、路径、内部token或研发配置；平台和企业DTO白名单分离</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J64"/>
+  <autoFilter ref="A1:J65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9633,7 +9685,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -13133,7 +13185,7 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>以现有63项导航处置矩阵重组企业Gateway：默认折叠并保持单组展开；首页按角色显示下一步任务；保留BYOK、Provider/模型/路由/评测、Project/Application、Virtual Key、额度预算、用量成本、企业内部财务、员工权限、安全策略、日志审计、Prompt、文件与文件安全、企业异步批处理、MCP、数据生命周期和私有部署；competitor-comparison移出产品UI；debug、intent测试、Webhook死信、环境诊断等仅高级角色按需进入。</t>
+          <t>以现有64项导航处置矩阵重组企业Gateway：默认折叠并保持单组展开；首页按角色显示下一步任务；保留BYOK、Provider/模型/路由/评测、Project/Application、Virtual Key、额度预算、用量成本、企业内部财务、员工权限、安全策略、日志审计、Prompt、文件与文件安全、企业异步批处理、MCP、数据生命周期和私有部署；competitor-comparison移出产品UI；debug、intent测试、Webhook死信、环境诊断等仅高级角色按需进入。</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
@@ -13173,7 +13225,7 @@
       </c>
       <c r="Q58" s="3" t="inlineStr">
         <is>
-          <t>63项现状导航每项有唯一处置且源码清单无遗漏；所有企业角色只看职责相关页；默认折叠、单组展开、直达URL负测试、真人鼠标主流程、390/1280/1440布局和无研发术语通过；每页只加载当前数据。</t>
+          <t>64项现状导航每项有唯一处置且源码清单无遗漏；所有企业角色只看职责相关页；默认折叠、单组展开、直达URL负测试、真人鼠标主流程、390/1280/1440布局和无研发术语通过；每页只加载当前数据。</t>
         </is>
       </c>
       <c r="R58" s="3" t="inlineStr">
@@ -13265,7 +13317,7 @@
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>按63项导航处置矩阵对代码、API、权限、表、事件、Scheduler、导航、DOM、文案、遥测和审计执行expand/dual-read/backfill/cutover/contract。盘点control_background_schedulers_enabled当前统一开关下安装的23个后台循环，逐个迁移执行身份、queue owner、lease和水位；Web副本不重复承担无界Worker。平台接管运营、品牌、Provider工程和商业目录；企业保留AI治理；拆分页使用独立主体；退役页面设置固定tombstone，不直接删除历史tenant_id事实。</t>
+          <t>按64项导航处置矩阵对代码、API、权限、表、事件、Scheduler、导航、DOM、文案、遥测和审计执行expand/dual-read/backfill/cutover/contract。盘点control_background_schedulers_enabled当前统一开关下安装的23个后台循环，逐个迁移执行身份、queue owner、lease和水位；Web副本不重复承担无界Worker。平台接管运营、品牌、Provider工程和商业目录；企业保留AI治理；拆分页使用独立主体；退役页面设置固定tombstone，不直接删除历史tenant_id事实。</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
@@ -13439,7 +13491,7 @@
       </c>
       <c r="Q60" s="3" t="inlineStr">
         <is>
-          <t>PRD-090..147全部完成；63项导航处置落地；平台/企业/伙伴/支持/设备五域负测试通过；WB/API/BB/GR/PERF/WEB/UI/UCD/COMP/SEC/FLOW全组通过；72小时无P0/P1；README/Excel/docs/HEAD/origin一致。</t>
+          <t>PRD-090..147全部完成；64项导航处置落地；平台/企业/伙伴/支持/设备五域负测试通过；WB/API/BB/GR/PERF/WEB/UI/UCD/COMP/SEC/FLOW全组通过；72小时无P0/P1；README/Excel/docs/HEAD/origin一致。</t>
         </is>
       </c>
       <c r="R60" s="3" t="inlineStr">
@@ -13826,7 +13878,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>G7通过；63项导航唯一处置、历史保真、企业旧平台入口归零</t>
+          <t>G7通过；64项导航唯一处置、历史保真、企业旧平台入口归零</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -45093,7 +45145,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>源码63项导航处置100%；平台运营/品牌/Provider工程/商业账务分域；历史行数/hash/outbox/Scheduler/审计水位保真；企业旧平台入口、DOM、预取/API归零</t>
+          <t>源码64项导航处置100%；平台运营/品牌/Provider工程/商业账务分域；历史行数/hash/outbox/Scheduler/审计水位保真；企业旧平台入口、DOM、预取/API归零</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-121 desired state
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..120已完成，下一项PRD-121。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..121已完成，下一项PRD-122。</t>
         </is>
       </c>
     </row>
@@ -9818,7 +9818,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-122 telemetry sync
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..121已完成，下一项PRD-122。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..122已完成，下一项PRD-123。</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-123 local secret custody
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..122已完成，下一项PRD-123。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..123已完成，下一项PRD-124。</t>
         </is>
       </c>
     </row>
@@ -10082,7 +10082,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-124 installer onboarding
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..123已完成，下一项PRD-124。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..124已完成，下一项PRD-125。</t>
         </is>
       </c>
     </row>
@@ -10215,7 +10215,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-127 fleet staged upgrades
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..126已完成，下一项PRD-127。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..127已完成，下一项PRD-128。</t>
         </is>
       </c>
     </row>
@@ -10612,7 +10612,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-128 license capacity
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..127已完成，下一项PRD-128。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..128已完成，下一项PRD-129。</t>
         </is>
       </c>
     </row>
@@ -10746,7 +10746,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-129 backup restore drills
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..128已完成，下一项PRD-129。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..129已完成，下一项PRD-130。</t>
         </is>
       </c>
     </row>
@@ -10879,7 +10879,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(edge): complete PRD-130 offline bundle reconciliation
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..129已完成，下一项PRD-130。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..130已完成，下一项PRD-131。</t>
         </is>
       </c>
     </row>
@@ -11012,7 +11012,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(migration): complete PRD-131 cutover operations
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..130已完成，下一项PRD-131。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..131已完成，下一项PRD-132。</t>
         </is>
       </c>
     </row>
@@ -11144,7 +11144,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(support): complete PRD-132 customer support
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..131已完成，下一项PRD-132。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..132已完成，下一项PRD-133。</t>
         </is>
       </c>
     </row>
@@ -11278,7 +11278,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: add public API and SDK lifecycle governance (PRD-133)
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..132已完成，下一项PRD-133。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..133已完成，下一项PRD-134。</t>
         </is>
       </c>
     </row>
@@ -11410,7 +11410,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(privacy): complete global account DSR center (PRD-134)
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..133已完成，下一项PRD-134。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..134已完成，下一项PRD-135。</t>
         </is>
       </c>
     </row>
@@ -11543,7 +11543,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(compliance): complete evidence center (PRD-135)
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..134已完成，下一项PRD-135。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..135已完成，下一项PRD-136。</t>
         </is>
       </c>
     </row>
@@ -11675,7 +11675,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(supply-chain): complete release security (PRD-136)
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..135已完成，下一项PRD-136。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..136已完成，下一项PRD-137。</t>
         </is>
       </c>
     </row>
@@ -11807,7 +11807,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(security): complete tenant isolation assurance (PRD-137)
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..136已完成，下一项PRD-137。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..137已完成，下一项PRD-138。</t>
         </is>
       </c>
     </row>
@@ -11939,7 +11939,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat: complete PRD-138 launch governance
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..137已完成，下一项PRD-138。</t>
+          <t>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..138已完成，下一项PRD-139。</t>
         </is>
       </c>
     </row>
@@ -12070,7 +12070,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>未启动</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
feat(customer-success): deliver platform renewal operations
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R64bb2c79b3724e59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="Rfee5d2c0905a4eab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Rf8303728f1cf4f42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Rdd60e6766d8c4d57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Re8493e0572ff4d3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R818012bc057e4d6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Ra7838a5356424bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R8b6c2c9acbe64ff1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R55affd35cffe4b55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R51ffb1d324394f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Re80e50c34b3d4c62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R324f2b1ad4ab4810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rac5dd899cc904de8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R01202a715a5d4450"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Re1608f03f7954cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R11e4c47c67e640a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rcce441d4135f48e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Re5a72eba047845c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rbb1718ba1ea94ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R7465468275ee46fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R3664c4baa4be4a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Re72ec8c2e7404f9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Ra59e612c5af24651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R2dcde77f2fef4b82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..139已完成，下一项PRD-140。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..140已完成，下一项PRD-141。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -12208,10 +12208,8 @@
           <x:t xml:space="preserve">PRD-140</x:t>
         </x:is>
       </x:c>
-      <x:c r="B52" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B52" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C52" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
feat: deliver PRD-141 platform growth analytics
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rac5dd899cc904de8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R01202a715a5d4450"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Re1608f03f7954cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R11e4c47c67e640a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rcce441d4135f48e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Re5a72eba047845c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rbb1718ba1ea94ad1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R7465468275ee46fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R3664c4baa4be4a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Re72ec8c2e7404f9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Ra59e612c5af24651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R2dcde77f2fef4b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R06be0fb7952d40f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R39cbe3a0f11c4a06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R78f68893b6864837"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Rb98cfbb98bf24b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R87201ba0249344e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Rff777d4fa6844d16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rcfb1392baea64895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="Rcf35237fcaf34d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R357755051f404572"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R65ab2760129f40da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R723397d426f545e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="Rc4184d1ad8f04963"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..140已完成，下一项PRD-141。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..141已完成，下一项PRD-142。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -12340,10 +12340,8 @@
           <x:t xml:space="preserve">PRD-141</x:t>
         </x:is>
       </x:c>
-      <x:c r="B53" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B53" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C53" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
feat(branding): deliver PRD-142 brand domains
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R06be0fb7952d40f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R39cbe3a0f11c4a06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R78f68893b6864837"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Rb98cfbb98bf24b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R87201ba0249344e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Rff777d4fa6844d16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rcfb1392baea64895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="Rcf35237fcaf34d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R357755051f404572"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R65ab2760129f40da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R723397d426f545e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="Rc4184d1ad8f04963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R77cac4b140fa472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R0dc41c84753c4145"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R4855061cfde74634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R81227b6ccf2045ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rb10c5a06a84c46d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R6eabba15f009452c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rff29055813d44925"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="Rc3a42042d86d4a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R57293fa79cfb4e73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R96eb75f0b08b4f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rfd4563f088fd4215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R34e6ad1ddd234178"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..141已完成，下一项PRD-142。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..142已完成，下一项PRD-143。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -12472,10 +12472,8 @@
           <x:t xml:space="preserve">PRD-142</x:t>
         </x:is>
       </x:c>
-      <x:c r="B54" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B54" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C54" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
feat(provider-engineering): deliver PRD-143 domains
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R77cac4b140fa472c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R0dc41c84753c4145"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R4855061cfde74634"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R81227b6ccf2045ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rb10c5a06a84c46d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R6eabba15f009452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rff29055813d44925"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="Rc3a42042d86d4a49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R57293fa79cfb4e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R96eb75f0b08b4f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rfd4563f088fd4215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R34e6ad1ddd234178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Ra759a73c26bf479e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R3b4d3c9bdf044dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Rfa5f07e1d1b14ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R8679731bad8140a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Re9961c636cd249f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R9041d03756484a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R8a486bdba54b4556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R11354e4710434ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R18d053ffbc8f4eaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R74b13362eb4347c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R3b039e6ff3dd4628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R94de466ebb9d4b96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..142已完成，下一项PRD-143。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..143已完成，下一项PRD-144。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -12603,10 +12603,8 @@
           <x:t xml:space="preserve">PRD-143</x:t>
         </x:is>
       </x:c>
-      <x:c r="B55" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B55" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C55" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
feat(commercial-accounting): deliver PRD-144 domain
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Ra759a73c26bf479e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R3b4d3c9bdf044dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Rfa5f07e1d1b14ebf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R8679731bad8140a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Re9961c636cd249f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R9041d03756484a5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R8a486bdba54b4556"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R11354e4710434ed0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R18d053ffbc8f4eaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R74b13362eb4347c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R3b039e6ff3dd4628"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R94de466ebb9d4b96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R47703a60e27f4714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R8b1ae693ec8b4d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R96eca7b8039e4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R7c7778e4bed0438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R5f0cf32c623d4777"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Rd69dc284851344b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rc5cb9153156845f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R21d3e38967cc4fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R4140185e03e34985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Rcabd12c2b38a43b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rd29432c7cecf45a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="Rc67f4f18eb6c4ed6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..143已完成，下一项PRD-144。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..144已完成，下一项PRD-145。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -12734,10 +12734,8 @@
           <x:t xml:space="preserve">PRD-144</x:t>
         </x:is>
       </x:c>
-      <x:c r="B56" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B56" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C56" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
feat(prd-145): split platform and workspace console experience
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R47703a60e27f4714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R8b1ae693ec8b4d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R96eca7b8039e4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R7c7778e4bed0438b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R5f0cf32c623d4777"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Rd69dc284851344b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rc5cb9153156845f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R21d3e38967cc4fa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R4140185e03e34985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="Rcabd12c2b38a43b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rd29432c7cecf45a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="Rc67f4f18eb6c4ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R82ef92b78db94a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R2b6180e4dfda403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R23dcdc08fc444285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Ra3ec45c5026a421b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R78d96374833f4b49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R00e7278bfdff42bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R4db231eadbb047ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R9bed2f393daf4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R0c3a0260669f438c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R97d8ec3fb6394e0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R4dc547e900df476f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R69d4e560aa954f75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -12868,10 +12868,8 @@
           <x:t xml:space="preserve">PRD-145</x:t>
         </x:is>
       </x:c>
-      <x:c r="B57" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B57" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C57" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
feat(prd-146): deliver workspace navigation and task home
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R82ef92b78db94a9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R2b6180e4dfda403f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R23dcdc08fc444285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Ra3ec45c5026a421b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R78d96374833f4b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R00e7278bfdff42bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R4db231eadbb047ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R9bed2f393daf4c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R0c3a0260669f438c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R97d8ec3fb6394e0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R4dc547e900df476f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R69d4e560aa954f75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rc35b1edb065c495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R1b28908f205d4558"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R6056d875b226423f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R22d3833ddeee420a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rd47234083ec14e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Rdd8b56a3fc414c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R18fc9c3de201407f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R0321793042cf43c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R6ad945780a464fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R3ef7f5f3feba4f94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R8b1731da60624f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R4ec0a838e4f64628"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13003,10 +13003,8 @@
           <x:t xml:space="preserve">PRD-146</x:t>
         </x:is>
       </x:c>
-      <x:c r="B58" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B58" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C58" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
docs(roadmap): close PRD-147 delivery
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rc35b1edb065c495e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R1b28908f205d4558"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R6056d875b226423f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R22d3833ddeee420a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rd47234083ec14e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Rdd8b56a3fc414c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R18fc9c3de201407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R0321793042cf43c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R6ad945780a464fea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R3ef7f5f3feba4f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R8b1731da60624f14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R4ec0a838e4f64628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rfa2c5606aef148da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="Rb016899674114404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R4fec6e75b3d4444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Ra7243af2d87e4de4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R248bfbb46ff84783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R9451ac55382544f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R317c9174a3514a75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R319707f56f554e4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R3286ed95b7ed4742"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R16576c5d82744846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R270cc2e3966b4f1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R8e52e184329d450d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..144已完成，下一项PRD-145。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..147已完成；G7未通过，PRD-148不得开始。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -13133,10 +13133,8 @@
           <x:t xml:space="preserve">PRD-147</x:t>
         </x:is>
       </x:c>
-      <x:c r="B59" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未启动</x:t>
-        </x:is>
+      <x:c r="B59" s="3" t="str">
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="C59" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
fix(g7): complete native database and cross-platform acceptance
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rfa2c5606aef148da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="Rb016899674114404"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="R4fec6e75b3d4444a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Ra7243af2d87e4de4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="R248bfbb46ff84783"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R9451ac55382544f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R317c9174a3514a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R319707f56f554e4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R3286ed95b7ed4742"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R16576c5d82744846"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R270cc2e3966b4f1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R8e52e184329d450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rb963afd9481e4104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="Rfbb2fd4117fa4d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Ra7d6d92f3bc14b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Ra8dbe04b3d814bcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rd01dccbdfa614196"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R34a9669ad53943cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rfeb2c6bc90424e56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="Rba988ef8e8e64e00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R2a5b4bec899f4424"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R79e85458fb8b46b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rc3c28563ed104cbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R0155f0b4fab84bb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；兼容旧状态all_108_prds_complete=false；PRD-090..147已完成；G7未通过，PRD-148不得开始。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；all_108_prds_complete=false；PRD-090..147实现完成，G7通过；G6缺72小时观测，PRD-148未启动。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">

</xml_diff>

<commit_message>
fix(prd138): serialize native launch governance and record observation interruption
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rb963afd9481e4104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="Rfbb2fd4117fa4d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Ra7d6d92f3bc14b8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="Ra8dbe04b3d814bcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rd01dccbdfa614196"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R34a9669ad53943cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rfeb2c6bc90424e56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="Rba988ef8e8e64e00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R2a5b4bec899f4424"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R79e85458fb8b46b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rc3c28563ed104cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R0155f0b4fab84bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R8e9069ceebf04dae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R28e71eecd84d44a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Rffe52f200c114190"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R52e4f618e6874abe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rbe2171a25ab44d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R9d9d034524ac40ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rcdda437450b84110"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R87ba0941e9b14b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R508b5ca5d0f24425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R355b67ce237e4923"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rd0631111cf844010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R9dcc7e6799e74cee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；all_108_prds_complete=false；PRD-090..147实现完成，G7通过；G6缺72小时观测，PRD-148未启动。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；all_108_prds_complete=false；PRD-090..147已有交付，G7通过；G6补实现、原生业务及72小时真实证据，PRD-148未启动。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">

</xml_diff>

<commit_message>
chore: publish current MetaHub development snapshot
</commit_message>
<xml_diff>
--- a/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
+++ b/企业级AI_Gateway_SaaS增量开发计划_PRD090起.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="R8e9069ceebf04dae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R28e71eecd84d44a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Rffe52f200c114190"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R52e4f618e6874abe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Rbe2171a25ab44d37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="R9d9d034524ac40ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="Rcdda437450b84110"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="R87ba0941e9b14b78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R508b5ca5d0f24425"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R355b67ce237e4923"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="Rd0631111cf844010"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="R9dcc7e6799e74cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_变更说明" sheetId="1" r:id="Rec17cac352c04a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_PRD总表" sheetId="2" r:id="R1d807fc06b734ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_阶段路线图" sheetId="3" r:id="Rcf6212f6fc2d43ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_核心数据对象" sheetId="4" r:id="R1ae7beff4ae9492a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_API与事件" sheetId="5" r:id="Ra278a458c0db4ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_角色权限矩阵" sheetId="6" r:id="Rf93a810891eb4b70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_测试与验收计划" sheetId="7" r:id="R5b47cef0194c42a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_旧计划废弃映射" sheetId="8" r:id="Rcc86d3f6d5a946a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_里程碑门禁" sheetId="9" r:id="R3e2f8e58bda349be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_风险与决策" sheetId="10" r:id="R9866fafe8f254c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_角色页面矩阵" sheetId="11" r:id="R51046280cffa4a43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_现有导航处置" sheetId="12" r:id="Ra4e58e5982464dbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -467,14 +467,18 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="5" ht="38" customHeight="1">
+    <x:row r="5" ht="72" customHeight="1">
       <x:c r="A5" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">总体状态</x:t>
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>saas_incremental_roadmap_complete=false；all_108_prds_complete=false；PRD-090..147已有交付，G7通过；G6补实现、原生业务及72小时真实证据，PRD-148未启动。</x:v>
+        <x:v>saas_incremental_roadmap_complete=false；all_108_prds_complete=false；2026-09-19 PRD-148：源码 bdb3204a...bb838（2689 文件）；page-visit 7/7。真实浏览器组织链未形成通过，保留 Chromium 登出 15 秒失败、page-visit 待完成和浏览器上下文异常；验收夹具查询参数错配已修正。五域、付费/治理、会签/回滚、对账、259200 秒稳定性和 HEAD/origin 未闭合，PRD-148 保持未启动。证据：outputs/prd148-current-evidence-index-final-20260916.json。；2026-09-20 current acceptance checkpoint: 当前源码 SHA256 6713a21a301d9b7cfb526df7dcf5b53e98dfd79a82d869ef08a14c86d17c0392（2691 files）；分批角色走查 admin/developer/viewer 180/180 页通过，证据 .artifacts/product-qa/20260920-{admin,developer,viewer}-g{1,2,3}；Workspace page-visit 集成 7/7 通过，证据 outputs/prd148-page-visits-current-20260920-r2.xml。真实 S1 当前重放 outputs/prd148-real-s1-rerun-20260920.json / .artifacts/s1-browser-_dluz246 仍失败于 1280.onboarding-navigation.tenant：截图等待字体超时，6 个 page-view 请求未结束；注册、创建组织、Provider、邀请员工、个人 KEY、轮换、撤权及撤权后 401 已完成，但完整商业链路不能宣称通过。五域矩阵已有 113/113 通过且起止源码漂移，不能绑定当前源码；真实商业、六方会签、发布后复核、回滚、财务/隐私/安全/迁移对账、scheduler-enabled 259200 秒观察及 HEAD/origin 一致仍未闭合。PRD-148 保持未完成，01_PRD总表!B60 保持未启动。
+2026-09-20 当前源码多角色批量走查：admin/developer/viewer Workspace 180/180 页，FLOW-01/02/03，Platform 运营迁移/MFA，公共入口四视口通过；Partner 浏览器验收在页面操作前因旧 0080 迁移基线夹具与当前 0155 迁移头漂移失败，未计 Partner 通过。前端 Partner/Support 21/21、后端 10/10 聚焦回归通过。证据 outputs/prd148-human-role-batch-current-20260920-r3.json；PRD-148 仍未启动。
+2026-09-20 Partner 当前页面边界复验：隔离 Chromium 390x844 在无 ChannelMembership 账号下连续两次返回 403 partner.membership_required，页面访问撤销态、布局和错误边界通过；函数序列化属于夹具问题；正常 Workspace 进入 Partner 的混合 Cookie 冲突已复现为真实入口失败，尚未修复。旧 PRD-087 浏览器验收仍受 0080→0155 迁移基线漂移阻断。证据 .artifacts/product-qa/20260920-partner-r7/prd148-partner-audit-chromium-scale-1.json；PRD-148 仍未启动。
+2026-09-20 有数据复核：Support 空页面已修复，管理员/开发者表单创建、回复、升级、解决、评价、重开和持久化通过，查看者写入 403。Device 空页面、Partner 入口 400 仍失败。旧 human-r4 聚合漏算断言，撤回完整交互通过结论。Support/Device 后端 24/24，Support 前端 8/8。详见 docs/testing/PRD-148-populated-domain-audit-20260920.md；完整 QA、真实商业及会签/对账/72小时/HEAD-origin 门禁未闭合，PRD-148 未启动。
+2026-09-24 当前成员撤权与角色化后台复核：成员移除会在同一事务停用个人 KEY、管理员分配 KEY、历史使用者关联和活动 Workspace session，旧凭据的 Gateway 鉴权立即拒绝；成员/使用者 9/9、Virtual Key 6/6、员工跨协议身份计量停用 1/1、Console 角色与 KEY 287/287 通过。当前源码 SHA256 0ff3be1ea56fee196b21ce6b20ff00f6c144429034956833a426e59aa0182d4f，生产资源摘要 be5564c28378fe2ab5e2d73c5c7bcd8efab194d4c87444c5010abb0bf2d2d87f。Gateway 宽集成因迁移夹具性能未形成 JUnit 终态；局部回归、本地健康和短时运行不构成 GA。按用户决定不执行 72 小时稳定性观察和六方会签，PRD-148 保持未完成。证据：outputs/prd148-member-key-current-20260924.json。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
@@ -12075,8 +12079,10 @@
           <x:t xml:space="preserve">PRD-139</x:t>
         </x:is>
       </x:c>
-      <x:c r="B51" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B51" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C51" s="3" t="inlineStr">
         <x:is>
@@ -12208,8 +12214,10 @@
           <x:t xml:space="preserve">PRD-140</x:t>
         </x:is>
       </x:c>
-      <x:c r="B52" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B52" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C52" s="3" t="inlineStr">
         <x:is>
@@ -12340,8 +12348,10 @@
           <x:t xml:space="preserve">PRD-141</x:t>
         </x:is>
       </x:c>
-      <x:c r="B53" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B53" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C53" s="3" t="inlineStr">
         <x:is>
@@ -12472,8 +12482,10 @@
           <x:t xml:space="preserve">PRD-142</x:t>
         </x:is>
       </x:c>
-      <x:c r="B54" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B54" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C54" s="3" t="inlineStr">
         <x:is>
@@ -12603,8 +12615,10 @@
           <x:t xml:space="preserve">PRD-143</x:t>
         </x:is>
       </x:c>
-      <x:c r="B55" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B55" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C55" s="3" t="inlineStr">
         <x:is>
@@ -12734,8 +12748,10 @@
           <x:t xml:space="preserve">PRD-144</x:t>
         </x:is>
       </x:c>
-      <x:c r="B56" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B56" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C56" s="3" t="inlineStr">
         <x:is>
@@ -12868,8 +12884,10 @@
           <x:t xml:space="preserve">PRD-145</x:t>
         </x:is>
       </x:c>
-      <x:c r="B57" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B57" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C57" s="3" t="inlineStr">
         <x:is>
@@ -13003,8 +13021,10 @@
           <x:t xml:space="preserve">PRD-146</x:t>
         </x:is>
       </x:c>
-      <x:c r="B58" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B58" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C58" s="3" t="inlineStr">
         <x:is>
@@ -13133,8 +13153,10 @@
           <x:t xml:space="preserve">PRD-147</x:t>
         </x:is>
       </x:c>
-      <x:c r="B59" s="3" t="str">
-        <x:v>已完成</x:v>
+      <x:c r="B59" s="3" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已完成</x:t>
+        </x:is>
       </x:c>
       <x:c r="C59" s="3" t="inlineStr">
         <x:is>
@@ -13385,10 +13407,26 @@
           <x:t xml:space="preserve">后端2、前端1、测试1；按领域增加SRE/安全/财务/Agent 0.5-1</x:t>
         </x:is>
       </x:c>
-      <x:c r="Y60" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">设计文档、两轮编码前自审、迁移往返、专项测试、必要回归、真实 API/浏览器/运行验收、安全与禁止文件审计</x:t>
-        </x:is>
+      <x:c r="Y60" s="3" t="str">
+        <x:v>2026-09-15 当前源码复核：Platform 38/38、Workspace 62/62、Partner/Support 16 通过+1 退役路由 skipped、Device 14/14；GA/Gateway 40/40；源码 SHA256 4a8f9efb…700b08c2。外部付费/企业治理/私有 Gateway、六方会签/回滚/对账、正式 scheduler-enabled 72 小时仍缺证据。PRD-148 未完成。索引 outputs/prd148-current-evidence-index-after-cache-20260915.json。
+2026-09-15 迁移实况复核：PRD-148 未完成。本机入口 expanded/generation 0，分域迁移、对账、审批和退役记录均为空。64 条队列契约不能证明导航迁移完成。新源码 QA 仍运行中，10 处旧迁移基线和 PRD-147 历史子集修复仅已准备候选、未应用。真实商业、会签、发布回滚、对账、72 小时和 HEAD/origin 仍缺证据。详见 docs/testing/PRD-148-current.md 及 outputs/prd148-console-migration-audit-20260915.json。以下为历史记录。
+2026-09-15：PRD-148 未完成。修复 0155 回滚入口拒绝问题，GA 回归 14/14；副本往返保留 1094 表、543694 行。修复前 QA 15/15 任务、审计 95/97，PERF-08/10 缺长稳。新源码 9904e348…cebfe 的完整 QA 与五域回归运行中。真实商业/会签/发布回滚/对账、72 小时及 HEAD/origin 仍未闭合。见 docs/testing/PRD-148-current.md。以下为历史记录。
+2026-09-15 复核更正：PRD-148 未完成。五域选定用例及 Gateway 回归通过；4/4 仅 QA 合同，完整 QA 补跑中。formal10 已停止、GA 计入 0 秒；健康接口不能证明业务 72 小时及 0 P0/P1。当前结论见 docs/testing/PRD-148-current.md；下方保留历史记录。
+2026-09-15 正式观察已按 scheduler-enabled 配置启动：formal10 当前运行中，必须达到 259200 秒且 0 P0/P1，运行中不计为通过。详见 outputs/continuous-stability-20260915-formal10/status.json。
+2026-09-15 正式观察已按 scheduler-enabled 配置启动：formal9 当前运行 56.72 秒、354 请求、0 错误；必须达到 259200 秒且 0 P0/P1，运行中不计为通过。详见 outputs/continuous-stability-20260915-formal9/status.json。
+2026-09-15 当前：五域负向矩阵 112 passed + 1 retired skipped；Gateway 协议 27/27；11 组 QA 合同 4/4 任务通过，源码 SHA256 da72cabf…571e7a。真实浏览器矩阵/兼容性终验、真实付费/会签/回滚/对账、正式 72 小时、HEAD/origin 仍缺证据。PRD-148 未完成。索引 outputs/prd148-current-evidence-index-20260915.json。
+设计文档、两轮编码前自审、迁移往返、专项测试、必要回归、真实 API/浏览器/运行验收、安全与禁止文件审计
+2026-09-14：未完成，当前证据见 docs/testing/PRD-148-current.md
+2026-09-14 当前证据追加：Platform 矩阵 38/38，健康/就绪 6/6；调度器开启 5 分钟诊断 0 错误（非 72 小时证据）；PRD-148 仍未完成。详见 outputs/prd148-negative-platform-current2-20260914.xml、outputs/continuous-stability-20260914-diagnostic3/status.json、docs/testing/PRD-148-current.md。
+2026-09-14 当前证据追加：Platform 矩阵 38/38，Platform 并发单项 1/1，健康/就绪 6/6；formal3 已失败（120 秒、7 个错误），formal4-isolated 已按调度器开启配置启动但仍未完成 72 小时；PRD-148 仍未完成。详见 outputs/prd148-negative-current2-20260914/status.json、outputs/prd148-platform-concurrency-followup-20260914.xml、outputs/continuous-stability-20260914-formal3/status.json、outputs/continuous-stability-20260914-formal4-isolated/status.json、docs/testing/PRD-148-current.md。
+2026-09-14 当前证据追加：Platform 矩阵 38/38，Platform 并发单项 1/1，健康/就绪 6/6；formal3 已失败（120 秒、7 个错误），formal4-isolated 亦已失败（372 秒、7 个 Control 超时），隔离数据库仍复现调度器争用；PRD-148 仍未完成。详见 outputs/prd148-negative-current2-20260914/status.json、outputs/prd148-platform-concurrency-followup-20260914.xml、outputs/continuous-stability-20260914-formal3/status.json、outputs/continuous-stability-20260914-formal4-isolated/status.json、docs/testing/PRD-148-current.md。
+2026-09-14 当前证据追加：共享 SQLite 连接按库一次启用 WAL；scheduler-enabled 诊断 120 秒 704 请求 0 错误，仍不构成 GA。正式 formal6 已按源码 SHA256 8471d7a5e254a2b8775b6a302faeaadb5216b6ad1be3dee99c18cf7fb182580e 启动，当前运行中，必须达到 259200 秒且 0 P0/P1。PRD-095 session P95 61.6ms（门槛 &lt;50ms）保留为真实失败；套餐/订阅/权益、付费计量、六方会签、发布回滚和最终对账仍缺证据。详见 docs/testing/PRD-148-current.md。
+2026-09-15 当前证据追加：修复 PRD-145 审批游标非规范 Base64url 接受问题，Workspace 44/44 与 GA 生命周期 13/13 通过；此前 Platform/Partner/Support/Device 证据早于该修复，需重新绑定当前源码。formal6 750.7 秒、3 次 Control read_timeout 失败；付费计划/订阅/权益/用量账本、真实六方会签/发布回滚/对账和 259200 秒正式观察仍缺，PRD-148 保持未完成。索引 outputs/prd148-current-evidence-index-20260915.json。
+2026-09-15 进一步修复：PRD-140 customer-success 游标同样拒绝非规范 Base64url；Platform 当前 38/38 通过。Partner/Support 与 Device 尚需最终源码快照重绑定；商业付费、会签/回滚/对账和 259200 秒正式观察仍未完成。
+2026-09-15 当前源码 QA 追加：All 5/5（WB/API/BB/GR/SEC、隔离 PERF、WEB/UI/UCD/COMP/FLOW、lint、Chromium admin/developer/viewer），PERF smoke/pressure 3/3；GA 14/14、协议/默认路由 24/24。formal11 运行约3531秒/0 errors，要求259200秒，不计为GA；付费订阅/权益、企业治理/私有Gateway、六方会签/回滚/对账和HEAD/origin仍缺证据。索引 outputs/prd148-current-evidence-index-final-20260915.json。
+2026-09-18 当前源码页面域审计 69/69；PAGE-116 Workspace Cookie 本地模型页修复；证据 outputs/prd148-domain-ui-audit-current-20260918-r4/report.json。PRD-148 未完成，见 outputs/prd148-current-evidence-index-final-20260916.json。
+2026-09-18 资源摘要同步后的当前源码页面域审计 69/69；PAGE-116 Workspace Cookie 本地模型页修复；源码 0143b226e96aac094667d32d03e2fe3aef590369c1cdb99aafc262f1e65d9384，生产摘要 aa58650f6c0b3c7badaaa4c69f5f05cd8717f54bec32ab3187c10894518f318b，证据 outputs/prd148-domain-ui-audit-current-20260918-r5/report.json。PRD-148 未完成，见 outputs/prd148-current-evidence-index-final-20260916.json。
+2026-09-24 当前成员撤权与角色化后台复核：成员移除会在同一事务停用个人 KEY、管理员分配 KEY、历史使用者关联和活动 Workspace session，旧凭据的 Gateway 鉴权立即拒绝；成员/使用者 9/9、Virtual Key 6/6、员工跨协议身份计量停用 1/1、Console 角色与 KEY 287/287 通过。当前源码 SHA256 0ff3be1ea56fee196b21ce6b20ff00f6c144429034956833a426e59aa0182d4f，生产资源摘要 be5564c28378fe2ab5e2d73c5c7bcd8efab194d4c87444c5010abb0bf2d2d87f。Gateway 宽集成因迁移夹具性能未形成 JUnit 终态；局部回归、本地健康和短时运行不构成 GA。按用户决定不执行 72 小时稳定性观察和六方会签，PRD-148 保持未完成。证据：outputs/prd148-member-key-current-20260924.json。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>